<commit_message>
#41 Control Board BOM LCSC MOQ Column Removed
</commit_message>
<xml_diff>
--- a/Deliverables/Control_Board/BOM/6 prototypes_Control_Board.xlsx
+++ b/Deliverables/Control_Board/BOM/6 prototypes_Control_Board.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25028"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ChrisitanRaun-AnnanasMotor\Deliverables\Control_Board\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ChristianRaun-EthercatDesign\Deliverables\Control_Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CCE9FDDE-E62A-4E79-A57C-9F68DA02A620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4374A5C1-953D-4F69-980F-F2BD06B94175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="175">
   <si>
     <t>S. No.</t>
   </si>
@@ -60,9 +60,6 @@
   </si>
   <si>
     <t>Value</t>
-  </si>
-  <si>
-    <t>LCSC/MOQ</t>
   </si>
   <si>
     <t>Quantity (Per Board)</t>
@@ -1054,7 +1051,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1198,9 +1195,6 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1210,19 +1204,7 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1231,9 +1213,6 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1297,9 +1276,6 @@
     <xf numFmtId="0" fontId="12" fillId="6" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1310,9 +1286,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1370,12 +1343,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="17" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1654,7 +1621,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="2" customWidth="1"/>
@@ -1667,32 +1634,30 @@
     <col min="8" max="8" width="14.42578125" style="2" customWidth="1"/>
     <col min="9" max="9" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="6.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5703125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="21.85546875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="14.140625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="9" style="1"/>
+    <col min="11" max="11" width="21.85546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="16.5" thickBot="1">
-      <c r="A1" s="96" t="s">
-        <v>161</v>
-      </c>
-      <c r="B1" s="97"/>
-      <c r="C1" s="97"/>
-      <c r="D1" s="97"/>
-      <c r="E1" s="97"/>
-      <c r="F1" s="97"/>
-      <c r="G1" s="97"/>
-      <c r="H1" s="97"/>
-      <c r="I1" s="97"/>
-      <c r="J1" s="97"/>
-      <c r="K1" s="97"/>
-      <c r="L1" s="97"/>
-      <c r="M1" s="97"/>
-      <c r="N1" s="97"/>
-    </row>
-    <row r="2" spans="1:15" ht="16.5" thickBot="1">
+    <row r="1" spans="1:14" ht="16.5" thickBot="1">
+      <c r="A1" s="88" t="s">
+        <v>160</v>
+      </c>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89"/>
+      <c r="H1" s="89"/>
+      <c r="I1" s="89"/>
+      <c r="J1" s="89"/>
+      <c r="K1" s="89"/>
+      <c r="L1" s="89"/>
+      <c r="M1" s="89"/>
+    </row>
+    <row r="2" spans="1:14" ht="16.5" thickBot="1">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -1727,1204 +1692,1124 @@
         <v>10</v>
       </c>
       <c r="L2" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="M2" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="N2" s="12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" ht="15.75" thickBot="1">
+    </row>
+    <row r="3" spans="1:14" ht="15.75" thickBot="1">
       <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="100" t="s">
+      <c r="B3" s="92" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="D3" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="52" t="s">
+      <c r="E3" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="F3" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="G3" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="26" t="s">
+      <c r="H3" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="27" t="s">
+      <c r="I3" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="28" t="s">
+      <c r="J3" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="18" t="s">
+      <c r="K3" s="29">
+        <v>4</v>
+      </c>
+      <c r="L3" s="29">
+        <f>K3*6</f>
+        <v>24</v>
+      </c>
+      <c r="M3" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="K3" s="29">
-        <v>25</v>
-      </c>
-      <c r="L3" s="29">
-        <v>4</v>
-      </c>
-      <c r="M3" s="29">
-        <f>L3*6</f>
-        <v>24</v>
-      </c>
-      <c r="N3" s="30" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" ht="39" thickBot="1">
+    </row>
+    <row r="4" spans="1:14" ht="39" thickBot="1">
       <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="101"/>
+      <c r="B4" s="93"/>
       <c r="C4" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="62" t="s">
+        <v>155</v>
+      </c>
+      <c r="E4" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="68" t="s">
-        <v>156</v>
-      </c>
-      <c r="E4" s="19" t="s">
+      <c r="F4" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="G4" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="32" t="s">
+      <c r="H4" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="33" t="s">
+      <c r="I4" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="I4" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="19" t="s">
-        <v>28</v>
-      </c>
       <c r="K4" s="34">
-        <v>150</v>
-      </c>
-      <c r="L4" s="34">
         <v>24</v>
       </c>
-      <c r="M4" s="29">
-        <f t="shared" ref="M4:M29" si="0">L4*6</f>
+      <c r="L4" s="29">
+        <f t="shared" ref="L4:L29" si="0">K4*6</f>
         <v>144</v>
       </c>
-      <c r="N4" s="35" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M4" s="35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="15.75" thickBot="1">
       <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="101"/>
+      <c r="B5" s="93"/>
       <c r="C5" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="36" t="s">
+      <c r="E5" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="14" t="s">
+      <c r="G5" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="G5" s="32" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5" s="33" t="s">
+      <c r="I5" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="I5" s="36" t="s">
+      <c r="J5" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="J5" s="19" t="s">
-        <v>34</v>
-      </c>
       <c r="K5" s="34">
-        <v>10</v>
-      </c>
-      <c r="L5" s="34">
         <v>1</v>
       </c>
-      <c r="M5" s="29">
+      <c r="L5" s="29">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="N5" s="35" t="s">
-        <v>22</v>
-      </c>
-      <c r="O5" s="13"/>
-    </row>
-    <row r="6" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M5" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="N5" s="13"/>
+    </row>
+    <row r="6" spans="1:14" ht="15.75" thickBot="1">
       <c r="A6" s="6">
         <v>4</v>
       </c>
-      <c r="B6" s="101"/>
+      <c r="B6" s="93"/>
       <c r="C6" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="36" t="s">
+      <c r="E6" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="F6" s="14" t="s">
+      <c r="G6" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="G6" s="32" t="s">
+      <c r="H6" s="33" t="s">
         <v>38</v>
       </c>
-      <c r="H6" s="33" t="s">
+      <c r="I6" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="I6" s="36" t="s">
+      <c r="J6" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="J6" s="19" t="s">
-        <v>41</v>
-      </c>
       <c r="K6" s="34">
-        <v>20</v>
-      </c>
-      <c r="L6" s="34">
         <v>3</v>
       </c>
-      <c r="M6" s="29">
+      <c r="L6" s="29">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="N6" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="O6" s="13"/>
-    </row>
-    <row r="7" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M6" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="N6" s="13"/>
+    </row>
+    <row r="7" spans="1:14" ht="15.75" thickBot="1">
       <c r="A7" s="6">
         <v>5</v>
       </c>
-      <c r="B7" s="102"/>
+      <c r="B7" s="94"/>
       <c r="C7" s="37" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="41" t="s">
+      <c r="E7" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="E7" s="38" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="15" t="s">
+      <c r="G7" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="G7" s="39" t="s">
+      <c r="H7" s="40" t="s">
         <v>45</v>
       </c>
-      <c r="H7" s="40" t="s">
+      <c r="I7" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="I7" s="41" t="s">
+      <c r="J7" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="J7" s="38" t="s">
-        <v>48</v>
-      </c>
       <c r="K7" s="42">
-        <v>100</v>
-      </c>
-      <c r="L7" s="42">
         <v>4</v>
       </c>
-      <c r="M7" s="29">
+      <c r="L7" s="29">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="N7" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="O7" s="13"/>
-    </row>
-    <row r="8" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M7" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="N7" s="13"/>
+    </row>
+    <row r="8" spans="1:14" ht="15.75" thickBot="1">
       <c r="A8" s="6">
         <v>6</v>
       </c>
       <c r="B8" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="D8" s="48" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="48" t="s">
+      <c r="E8" s="45" t="s">
         <v>51</v>
       </c>
-      <c r="E8" s="45" t="s">
+      <c r="F8" s="45" t="s">
         <v>52</v>
       </c>
-      <c r="F8" s="45" t="s">
+      <c r="G8" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="G8" s="46" t="s">
+      <c r="H8" s="47" t="s">
         <v>54</v>
       </c>
-      <c r="H8" s="47" t="s">
+      <c r="I8" s="48" t="s">
+        <v>19</v>
+      </c>
+      <c r="J8" s="46" t="s">
         <v>55</v>
       </c>
-      <c r="I8" s="48" t="s">
-        <v>20</v>
-      </c>
-      <c r="J8" s="46" t="s">
-        <v>56</v>
-      </c>
       <c r="K8" s="49">
-        <v>20</v>
-      </c>
-      <c r="L8" s="50">
         <v>3</v>
       </c>
-      <c r="M8" s="29">
+      <c r="L8" s="29">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="N8" s="51" t="s">
-        <v>22</v>
-      </c>
-      <c r="O8" s="13"/>
-    </row>
-    <row r="9" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M8" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="N8" s="13"/>
+    </row>
+    <row r="9" spans="1:14" ht="15.75" thickBot="1">
       <c r="A9" s="6">
         <v>7</v>
       </c>
-      <c r="B9" s="100" t="s">
+      <c r="B9" s="92" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="C9" s="25" t="s">
+      <c r="D9" s="51" t="s">
         <v>58</v>
       </c>
-      <c r="D9" s="52" t="s">
+      <c r="E9" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="F9" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="G9" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="G9" s="26" t="s">
+      <c r="H9" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="H9" s="27" t="s">
-        <v>63</v>
-      </c>
-      <c r="I9" s="52" t="s">
-        <v>20</v>
+      <c r="I9" s="51" t="s">
+        <v>19</v>
       </c>
       <c r="J9" s="26" t="s">
-        <v>56</v>
-      </c>
-      <c r="K9" s="53">
-        <v>50</v>
+        <v>55</v>
+      </c>
+      <c r="K9" s="29">
+        <v>5</v>
       </c>
       <c r="L9" s="29">
-        <v>5</v>
-      </c>
-      <c r="M9" s="29">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="N9" s="30" t="s">
-        <v>22</v>
-      </c>
-      <c r="O9" s="13"/>
-    </row>
-    <row r="10" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M9" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="N9" s="13"/>
+    </row>
+    <row r="10" spans="1:14" ht="15.75" thickBot="1">
       <c r="A10" s="6">
         <v>8</v>
       </c>
-      <c r="B10" s="102"/>
+      <c r="B10" s="94"/>
       <c r="C10" s="37" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="41" t="s">
         <v>64</v>
       </c>
-      <c r="D10" s="41" t="s">
+      <c r="E10" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="38" t="s">
+      <c r="F10" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="F10" s="38" t="s">
+      <c r="G10" s="39" t="s">
         <v>67</v>
       </c>
-      <c r="G10" s="39" t="s">
+      <c r="H10" s="40" t="s">
         <v>68</v>
       </c>
-      <c r="H10" s="40" t="s">
-        <v>69</v>
-      </c>
       <c r="I10" s="41" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J10" s="39" t="s">
-        <v>56</v>
-      </c>
-      <c r="K10" s="54">
-        <v>10</v>
-      </c>
-      <c r="L10" s="42">
+        <v>55</v>
+      </c>
+      <c r="K10" s="42">
         <v>1</v>
       </c>
-      <c r="M10" s="29">
+      <c r="L10" s="29">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="N10" s="55" t="s">
-        <v>22</v>
-      </c>
-      <c r="O10" s="13"/>
-    </row>
-    <row r="11" spans="1:15" ht="26.25" thickBot="1">
+      <c r="M10" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="N10" s="13"/>
+    </row>
+    <row r="11" spans="1:14" ht="26.25" thickBot="1">
       <c r="A11" s="6">
         <v>9</v>
       </c>
-      <c r="B11" s="100" t="s">
+      <c r="B11" s="92" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="D11" s="63" t="s">
         <v>71</v>
       </c>
-      <c r="D11" s="69" t="s">
+      <c r="E11" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="F11" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="G11" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="H11" s="27" t="s">
         <v>74</v>
       </c>
-      <c r="G11" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="H11" s="27" t="s">
+      <c r="I11" s="51" t="s">
+        <v>19</v>
+      </c>
+      <c r="J11" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="I11" s="52" t="s">
-        <v>20</v>
-      </c>
-      <c r="J11" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="K11" s="56">
-        <v>100</v>
+      <c r="K11" s="29">
+        <v>12</v>
       </c>
       <c r="L11" s="29">
-        <v>12</v>
-      </c>
-      <c r="M11" s="29">
         <f t="shared" si="0"/>
         <v>72</v>
       </c>
-      <c r="N11" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="O11" s="13"/>
-    </row>
-    <row r="12" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M11" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="N11" s="13"/>
+    </row>
+    <row r="12" spans="1:14" ht="15.75" thickBot="1">
       <c r="A12" s="6">
         <v>10</v>
       </c>
-      <c r="B12" s="101"/>
+      <c r="B12" s="93"/>
       <c r="C12" s="31" t="s">
+        <v>76</v>
+      </c>
+      <c r="D12" s="36" t="s">
         <v>77</v>
       </c>
-      <c r="D12" s="36" t="s">
+      <c r="E12" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="F12" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="E12" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="F12" s="19" t="s">
+      <c r="G12" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="G12" s="32" t="s">
-        <v>26</v>
-      </c>
-      <c r="H12" s="33" t="s">
+      <c r="I12" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="J12" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="I12" s="36" t="s">
-        <v>20</v>
-      </c>
-      <c r="J12" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="K12" s="57">
-        <v>100</v>
-      </c>
-      <c r="L12" s="34">
+      <c r="K12" s="34">
         <v>3</v>
       </c>
-      <c r="M12" s="29">
+      <c r="L12" s="29">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="N12" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="O12" s="13"/>
-    </row>
-    <row r="13" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M12" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="N12" s="13"/>
+    </row>
+    <row r="13" spans="1:14" ht="15.75" thickBot="1">
       <c r="A13" s="6">
         <v>11</v>
       </c>
-      <c r="B13" s="101"/>
+      <c r="B13" s="93"/>
       <c r="C13" s="31" t="s">
+        <v>81</v>
+      </c>
+      <c r="D13" s="36" t="s">
         <v>82</v>
       </c>
-      <c r="D13" s="36" t="s">
+      <c r="E13" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="F13" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="E13" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="F13" s="19" t="s">
+      <c r="G13" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="H13" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="G13" s="32" t="s">
-        <v>26</v>
-      </c>
-      <c r="H13" s="33" t="s">
+      <c r="I13" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="J13" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="I13" s="36" t="s">
-        <v>20</v>
-      </c>
-      <c r="J13" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="K13" s="57">
-        <v>100</v>
-      </c>
-      <c r="L13" s="34">
+      <c r="K13" s="34">
         <v>1</v>
       </c>
-      <c r="M13" s="29">
+      <c r="L13" s="29">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="N13" s="58" t="s">
-        <v>22</v>
-      </c>
-      <c r="O13" s="13"/>
-    </row>
-    <row r="14" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M13" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="N13" s="13"/>
+    </row>
+    <row r="14" spans="1:14" ht="15.75" thickBot="1">
       <c r="A14" s="6">
         <v>12</v>
       </c>
-      <c r="B14" s="101"/>
+      <c r="B14" s="93"/>
       <c r="C14" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="D14" s="36" t="s">
         <v>87</v>
       </c>
-      <c r="D14" s="36" t="s">
+      <c r="E14" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="F14" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="E14" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="F14" s="19" t="s">
+      <c r="G14" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="H14" s="33" t="s">
         <v>89</v>
       </c>
-      <c r="G14" s="32" t="s">
-        <v>26</v>
-      </c>
-      <c r="H14" s="33" t="s">
+      <c r="I14" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="J14" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="I14" s="36" t="s">
-        <v>20</v>
-      </c>
-      <c r="J14" s="19" t="s">
-        <v>91</v>
-      </c>
-      <c r="K14" s="57">
-        <v>100</v>
-      </c>
-      <c r="L14" s="34">
+      <c r="K14" s="34">
         <v>4</v>
       </c>
-      <c r="M14" s="29">
+      <c r="L14" s="29">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="N14" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="O14" s="13"/>
-    </row>
-    <row r="15" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M14" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="N14" s="13"/>
+    </row>
+    <row r="15" spans="1:14" ht="15.75" thickBot="1">
       <c r="A15" s="6">
         <v>13</v>
       </c>
-      <c r="B15" s="103"/>
-      <c r="C15" s="70" t="s">
+      <c r="B15" s="95"/>
+      <c r="C15" s="64" t="s">
+        <v>91</v>
+      </c>
+      <c r="D15" s="62" t="s">
         <v>92</v>
       </c>
-      <c r="D15" s="68" t="s">
+      <c r="E15" s="65" t="s">
+        <v>72</v>
+      </c>
+      <c r="F15" s="65" t="s">
         <v>93</v>
       </c>
-      <c r="E15" s="71" t="s">
-        <v>73</v>
-      </c>
-      <c r="F15" s="71" t="s">
+      <c r="G15" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="H15" s="33" t="s">
         <v>94</v>
       </c>
-      <c r="G15" s="32" t="s">
-        <v>26</v>
-      </c>
-      <c r="H15" s="33" t="s">
+      <c r="I15" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="J15" s="65" t="s">
         <v>95</v>
       </c>
-      <c r="I15" s="36" t="s">
-        <v>20</v>
-      </c>
-      <c r="J15" s="71" t="s">
-        <v>96</v>
-      </c>
-      <c r="K15" s="57">
-        <v>100</v>
-      </c>
-      <c r="L15" s="71">
+      <c r="K15" s="65">
         <v>2</v>
       </c>
-      <c r="M15" s="29">
+      <c r="L15" s="29">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="N15" s="72" t="s">
-        <v>22</v>
-      </c>
-      <c r="O15" s="13"/>
-    </row>
-    <row r="16" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M15" s="66" t="s">
+        <v>21</v>
+      </c>
+      <c r="N15" s="13"/>
+    </row>
+    <row r="16" spans="1:14" ht="15.75" thickBot="1">
       <c r="A16" s="6">
         <v>14</v>
       </c>
-      <c r="B16" s="103"/>
-      <c r="C16" s="70" t="s">
+      <c r="B16" s="95"/>
+      <c r="C16" s="64" t="s">
+        <v>96</v>
+      </c>
+      <c r="D16" s="62" t="s">
         <v>97</v>
       </c>
-      <c r="D16" s="68" t="s">
+      <c r="E16" s="65" t="s">
+        <v>72</v>
+      </c>
+      <c r="F16" s="65" t="s">
         <v>98</v>
       </c>
-      <c r="E16" s="71" t="s">
-        <v>73</v>
-      </c>
-      <c r="F16" s="71" t="s">
+      <c r="G16" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="H16" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="G16" s="32" t="s">
-        <v>26</v>
-      </c>
-      <c r="H16" s="33" t="s">
+      <c r="I16" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="J16" s="65" t="s">
         <v>100</v>
       </c>
-      <c r="I16" s="36" t="s">
-        <v>20</v>
-      </c>
-      <c r="J16" s="71" t="s">
-        <v>101</v>
-      </c>
-      <c r="K16" s="57">
-        <v>100</v>
-      </c>
-      <c r="L16" s="71">
+      <c r="K16" s="65">
         <v>1</v>
       </c>
-      <c r="M16" s="29">
+      <c r="L16" s="29">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="N16" s="72" t="s">
-        <v>22</v>
-      </c>
-      <c r="O16" s="13"/>
-    </row>
-    <row r="17" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M16" s="66" t="s">
+        <v>21</v>
+      </c>
+      <c r="N16" s="13"/>
+    </row>
+    <row r="17" spans="1:14" ht="15.75" thickBot="1">
       <c r="A17" s="6">
         <v>15</v>
       </c>
-      <c r="B17" s="102"/>
+      <c r="B17" s="94"/>
       <c r="C17" s="37" t="s">
+        <v>101</v>
+      </c>
+      <c r="D17" s="41" t="s">
         <v>102</v>
       </c>
-      <c r="D17" s="41" t="s">
+      <c r="E17" s="38" t="s">
+        <v>72</v>
+      </c>
+      <c r="F17" s="38" t="s">
         <v>103</v>
       </c>
-      <c r="E17" s="38" t="s">
-        <v>73</v>
-      </c>
-      <c r="F17" s="38" t="s">
+      <c r="G17" s="39" t="s">
         <v>104</v>
       </c>
-      <c r="G17" s="39" t="s">
+      <c r="H17" s="40" t="s">
         <v>105</v>
       </c>
-      <c r="H17" s="40" t="s">
+      <c r="I17" s="41" t="s">
+        <v>19</v>
+      </c>
+      <c r="J17" s="38" t="s">
         <v>106</v>
       </c>
-      <c r="I17" s="41" t="s">
-        <v>20</v>
-      </c>
-      <c r="J17" s="38" t="s">
-        <v>107</v>
-      </c>
       <c r="K17" s="42">
-        <v>100</v>
-      </c>
-      <c r="L17" s="42">
         <v>1</v>
       </c>
-      <c r="M17" s="29">
+      <c r="L17" s="29">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="N17" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="O17" s="13"/>
-    </row>
-    <row r="18" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M17" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="N17" s="13"/>
+    </row>
+    <row r="18" spans="1:14" ht="15.75" thickBot="1">
       <c r="A18" s="6">
         <v>16</v>
       </c>
       <c r="B18" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="C18" s="54" t="s">
         <v>108</v>
       </c>
-      <c r="C18" s="59" t="s">
+      <c r="D18" s="48" t="s">
         <v>109</v>
       </c>
-      <c r="D18" s="48" t="s">
+      <c r="E18" s="48" t="s">
         <v>110</v>
       </c>
-      <c r="E18" s="48" t="s">
+      <c r="F18" s="48" t="s">
         <v>111</v>
       </c>
-      <c r="F18" s="48" t="s">
+      <c r="G18" s="22" t="s">
         <v>112</v>
       </c>
-      <c r="G18" s="22" t="s">
-        <v>113</v>
-      </c>
       <c r="H18" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I18" s="48" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J18" s="22" t="s">
-        <v>56</v>
-      </c>
-      <c r="K18" s="60">
-        <v>10</v>
-      </c>
-      <c r="L18" s="50">
+        <v>55</v>
+      </c>
+      <c r="K18" s="49">
         <v>1</v>
       </c>
-      <c r="M18" s="29">
+      <c r="L18" s="29">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="N18" s="51" t="s">
-        <v>22</v>
-      </c>
-      <c r="O18" s="13"/>
-    </row>
-    <row r="19" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M18" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="N18" s="13"/>
+    </row>
+    <row r="19" spans="1:14" ht="15.75" thickBot="1">
       <c r="A19" s="6">
         <v>17</v>
       </c>
-      <c r="B19" s="100" t="s">
+      <c r="B19" s="92" t="s">
+        <v>113</v>
+      </c>
+      <c r="C19" s="67" t="s">
         <v>114</v>
       </c>
-      <c r="C19" s="73" t="s">
+      <c r="D19" s="68" t="s">
         <v>115</v>
       </c>
-      <c r="D19" s="74" t="s">
+      <c r="E19" s="69" t="s">
+        <v>161</v>
+      </c>
+      <c r="F19" s="68" t="s">
         <v>116</v>
       </c>
-      <c r="E19" s="75" t="s">
+      <c r="G19" s="71" t="s">
         <v>162</v>
       </c>
-      <c r="F19" s="74" t="s">
-        <v>117</v>
-      </c>
-      <c r="G19" s="77" t="s">
+      <c r="H19" s="72" t="s">
+        <v>157</v>
+      </c>
+      <c r="I19" s="72" t="s">
         <v>163</v>
       </c>
-      <c r="H19" s="78" t="s">
-        <v>158</v>
-      </c>
-      <c r="I19" s="78" t="s">
-        <v>164</v>
-      </c>
-      <c r="J19" s="78" t="s">
-        <v>56</v>
-      </c>
-      <c r="K19" s="77">
-        <v>5</v>
-      </c>
-      <c r="L19" s="75">
+      <c r="J19" s="72" t="s">
+        <v>55</v>
+      </c>
+      <c r="K19" s="69">
         <v>1</v>
       </c>
-      <c r="M19" s="29">
+      <c r="L19" s="29">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="N19" s="79" t="s">
-        <v>141</v>
-      </c>
-      <c r="O19" s="13"/>
-    </row>
-    <row r="20" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M19" s="73" t="s">
+        <v>140</v>
+      </c>
+      <c r="N19" s="13"/>
+    </row>
+    <row r="20" spans="1:14" ht="15.75" thickBot="1">
       <c r="A20" s="6">
         <v>18</v>
       </c>
-      <c r="B20" s="101"/>
-      <c r="C20" s="61" t="s">
+      <c r="B20" s="93"/>
+      <c r="C20" s="55" t="s">
+        <v>117</v>
+      </c>
+      <c r="D20" s="36" t="s">
         <v>118</v>
       </c>
-      <c r="D20" s="36" t="s">
+      <c r="E20" s="36" t="s">
         <v>119</v>
       </c>
-      <c r="E20" s="36" t="s">
+      <c r="F20" s="36" t="s">
         <v>120</v>
       </c>
-      <c r="F20" s="36" t="s">
+      <c r="G20" s="20" t="s">
         <v>121</v>
       </c>
-      <c r="G20" s="20" t="s">
+      <c r="H20" s="33" t="s">
         <v>122</v>
       </c>
-      <c r="H20" s="33" t="s">
-        <v>123</v>
-      </c>
       <c r="I20" s="36" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J20" s="20" t="s">
-        <v>56</v>
-      </c>
-      <c r="K20" s="33">
-        <v>6</v>
-      </c>
-      <c r="L20" s="34">
+        <v>55</v>
+      </c>
+      <c r="K20" s="34">
         <v>1</v>
       </c>
-      <c r="M20" s="29">
+      <c r="L20" s="29">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="N20" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="O20" s="13"/>
-    </row>
-    <row r="21" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M20" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="N20" s="13"/>
+    </row>
+    <row r="21" spans="1:14" ht="15.75" thickBot="1">
       <c r="A21" s="6">
         <v>19</v>
       </c>
-      <c r="B21" s="101"/>
-      <c r="C21" s="91" t="s">
+      <c r="B21" s="93"/>
+      <c r="C21" s="83" t="s">
+        <v>123</v>
+      </c>
+      <c r="D21" s="74" t="s">
         <v>124</v>
       </c>
-      <c r="D21" s="80" t="s">
+      <c r="E21" s="74" t="s">
+        <v>119</v>
+      </c>
+      <c r="F21" s="74" t="s">
         <v>125</v>
       </c>
-      <c r="E21" s="80" t="s">
-        <v>120</v>
-      </c>
-      <c r="F21" s="80" t="s">
+      <c r="G21" s="75" t="s">
         <v>126</v>
       </c>
-      <c r="G21" s="81" t="s">
-        <v>127</v>
-      </c>
-      <c r="H21" s="81" t="s">
-        <v>20</v>
-      </c>
-      <c r="I21" s="80" t="s">
-        <v>20</v>
-      </c>
-      <c r="J21" s="81" t="s">
-        <v>56</v>
-      </c>
-      <c r="K21" s="82">
-        <v>10</v>
-      </c>
-      <c r="L21" s="83">
+      <c r="H21" s="75" t="s">
+        <v>19</v>
+      </c>
+      <c r="I21" s="74" t="s">
+        <v>19</v>
+      </c>
+      <c r="J21" s="75" t="s">
+        <v>55</v>
+      </c>
+      <c r="K21" s="76">
         <v>1</v>
       </c>
-      <c r="M21" s="29">
+      <c r="L21" s="29">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="N21" s="84" t="s">
-        <v>146</v>
-      </c>
-      <c r="O21" s="13"/>
-    </row>
-    <row r="22" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M21" s="77" t="s">
+        <v>145</v>
+      </c>
+      <c r="N21" s="13"/>
+    </row>
+    <row r="22" spans="1:14" ht="15.75" thickBot="1">
       <c r="A22" s="6">
         <v>20</v>
       </c>
-      <c r="B22" s="102"/>
-      <c r="C22" s="92" t="s">
+      <c r="B22" s="94"/>
+      <c r="C22" s="84" t="s">
+        <v>127</v>
+      </c>
+      <c r="D22" s="78" t="s">
         <v>128</v>
       </c>
-      <c r="D22" s="85" t="s">
+      <c r="E22" s="78" t="s">
         <v>129</v>
       </c>
-      <c r="E22" s="85" t="s">
+      <c r="F22" s="78" t="s">
         <v>130</v>
       </c>
-      <c r="F22" s="85" t="s">
+      <c r="G22" s="78" t="s">
         <v>131</v>
       </c>
-      <c r="G22" s="85" t="s">
+      <c r="H22" s="78" t="s">
         <v>132</v>
       </c>
-      <c r="H22" s="85" t="s">
-        <v>133</v>
-      </c>
-      <c r="I22" s="85" t="s">
-        <v>20</v>
-      </c>
-      <c r="J22" s="86" t="s">
-        <v>56</v>
-      </c>
-      <c r="K22" s="87">
-        <v>10</v>
-      </c>
-      <c r="L22" s="88">
+      <c r="I22" s="78" t="s">
+        <v>19</v>
+      </c>
+      <c r="J22" s="79" t="s">
+        <v>55</v>
+      </c>
+      <c r="K22" s="80">
         <v>1</v>
       </c>
-      <c r="M22" s="29">
+      <c r="L22" s="29">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="N22" s="89" t="s">
-        <v>146</v>
-      </c>
-      <c r="O22" s="13"/>
-    </row>
-    <row r="23" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M22" s="81" t="s">
+        <v>145</v>
+      </c>
+      <c r="N22" s="13"/>
+    </row>
+    <row r="23" spans="1:14" ht="15.75" thickBot="1">
       <c r="A23" s="6">
         <v>21</v>
       </c>
-      <c r="B23" s="100" t="s">
+      <c r="B23" s="92" t="s">
+        <v>133</v>
+      </c>
+      <c r="C23" s="67" t="s">
         <v>134</v>
       </c>
-      <c r="C23" s="73" t="s">
+      <c r="D23" s="68" t="s">
         <v>135</v>
       </c>
-      <c r="D23" s="74" t="s">
+      <c r="E23" s="68" t="s">
+        <v>110</v>
+      </c>
+      <c r="F23" s="68" t="s">
         <v>136</v>
       </c>
-      <c r="E23" s="74" t="s">
-        <v>111</v>
-      </c>
-      <c r="F23" s="74" t="s">
-        <v>137</v>
-      </c>
-      <c r="G23" s="75" t="s">
-        <v>171</v>
-      </c>
-      <c r="H23" s="76"/>
-      <c r="I23" s="77"/>
-      <c r="J23" s="77"/>
-      <c r="K23" s="77"/>
-      <c r="L23" s="75">
+      <c r="G23" s="69" t="s">
+        <v>170</v>
+      </c>
+      <c r="H23" s="70"/>
+      <c r="I23" s="71"/>
+      <c r="J23" s="71"/>
+      <c r="K23" s="69">
         <v>1</v>
       </c>
-      <c r="M23" s="29">
+      <c r="L23" s="29">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="N23" s="23"/>
-      <c r="O23" s="13"/>
-    </row>
-    <row r="24" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M23" s="23"/>
+      <c r="N23" s="13"/>
+    </row>
+    <row r="24" spans="1:14" ht="15.75" thickBot="1">
       <c r="A24" s="6">
         <v>22</v>
       </c>
-      <c r="B24" s="102"/>
-      <c r="C24" s="92" t="s">
+      <c r="B24" s="94"/>
+      <c r="C24" s="84" t="s">
+        <v>137</v>
+      </c>
+      <c r="D24" s="78" t="s">
         <v>138</v>
       </c>
-      <c r="D24" s="85" t="s">
+      <c r="E24" s="78" t="s">
+        <v>110</v>
+      </c>
+      <c r="F24" s="78" t="s">
         <v>139</v>
       </c>
-      <c r="E24" s="85" t="s">
-        <v>111</v>
-      </c>
-      <c r="F24" s="85" t="s">
-        <v>140</v>
-      </c>
-      <c r="G24" s="85" t="s">
+      <c r="G24" s="78" t="s">
+        <v>157</v>
+      </c>
+      <c r="H24" s="78" t="s">
+        <v>19</v>
+      </c>
+      <c r="I24" s="78" t="s">
+        <v>157</v>
+      </c>
+      <c r="J24" s="78" t="s">
         <v>158</v>
       </c>
-      <c r="H24" s="85" t="s">
-        <v>20</v>
-      </c>
-      <c r="I24" s="85" t="s">
-        <v>158</v>
-      </c>
-      <c r="J24" s="85" t="s">
-        <v>159</v>
-      </c>
-      <c r="K24" s="87">
-        <v>7</v>
-      </c>
-      <c r="L24" s="88">
+      <c r="K24" s="80">
         <v>1</v>
       </c>
-      <c r="M24" s="29">
+      <c r="L24" s="29">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="N24" s="89" t="s">
-        <v>141</v>
-      </c>
-      <c r="O24" s="13"/>
-    </row>
-    <row r="25" spans="1:15" ht="39" customHeight="1" thickBot="1">
+      <c r="M24" s="81" t="s">
+        <v>140</v>
+      </c>
+      <c r="N24" s="13"/>
+    </row>
+    <row r="25" spans="1:14" ht="39" customHeight="1" thickBot="1">
       <c r="A25" s="6">
         <v>23</v>
       </c>
-      <c r="B25" s="104" t="s">
+      <c r="B25" s="96" t="s">
+        <v>141</v>
+      </c>
+      <c r="C25" s="86" t="s">
+        <v>164</v>
+      </c>
+      <c r="D25" s="82" t="s">
+        <v>166</v>
+      </c>
+      <c r="E25" s="82" t="s">
         <v>142</v>
       </c>
-      <c r="C25" s="94" t="s">
-        <v>165</v>
-      </c>
-      <c r="D25" s="90" t="s">
-        <v>167</v>
-      </c>
-      <c r="E25" s="90" t="s">
+      <c r="F25" s="82" t="s">
         <v>143</v>
       </c>
-      <c r="F25" s="90" t="s">
+      <c r="G25" s="82" t="s">
         <v>144</v>
       </c>
-      <c r="G25" s="90" t="s">
-        <v>145</v>
-      </c>
-      <c r="H25" s="90" t="s">
+      <c r="H25" s="82" t="s">
+        <v>157</v>
+      </c>
+      <c r="I25" s="82" t="s">
+        <v>19</v>
+      </c>
+      <c r="J25" s="82" t="s">
         <v>158</v>
       </c>
-      <c r="I25" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="J25" s="90" t="s">
-        <v>159</v>
-      </c>
-      <c r="K25" s="107">
-        <v>5</v>
-      </c>
-      <c r="L25" s="93">
+      <c r="K25" s="85">
         <v>2</v>
       </c>
-      <c r="M25" s="29">
+      <c r="L25" s="29">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="N25" s="105" t="s">
-        <v>146</v>
-      </c>
-      <c r="O25" s="13"/>
-    </row>
-    <row r="26" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M25" s="97" t="s">
+        <v>145</v>
+      </c>
+      <c r="N25" s="13"/>
+    </row>
+    <row r="26" spans="1:14" ht="15.75" thickBot="1">
       <c r="A26" s="6">
         <v>24</v>
       </c>
-      <c r="B26" s="104"/>
-      <c r="C26" s="91" t="s">
-        <v>166</v>
-      </c>
-      <c r="D26" s="90" t="s">
+      <c r="B26" s="96"/>
+      <c r="C26" s="83" t="s">
+        <v>165</v>
+      </c>
+      <c r="D26" s="82" t="s">
+        <v>168</v>
+      </c>
+      <c r="E26" s="74" t="s">
+        <v>167</v>
+      </c>
+      <c r="F26" s="74" t="s">
         <v>169</v>
       </c>
-      <c r="E26" s="80" t="s">
-        <v>168</v>
-      </c>
-      <c r="F26" s="80" t="s">
-        <v>170</v>
-      </c>
-      <c r="G26" s="80" t="s">
-        <v>145</v>
-      </c>
-      <c r="H26" s="90" t="s">
+      <c r="G26" s="74" t="s">
+        <v>144</v>
+      </c>
+      <c r="H26" s="82" t="s">
+        <v>157</v>
+      </c>
+      <c r="I26" s="82" t="s">
+        <v>163</v>
+      </c>
+      <c r="J26" s="82" t="s">
         <v>158</v>
       </c>
-      <c r="I26" s="90" t="s">
-        <v>164</v>
-      </c>
-      <c r="J26" s="90" t="s">
-        <v>159</v>
-      </c>
-      <c r="K26" s="108"/>
-      <c r="L26" s="93">
+      <c r="K26" s="85">
         <v>1</v>
       </c>
-      <c r="M26" s="29">
+      <c r="L26" s="29">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="N26" s="106"/>
-      <c r="O26" s="13"/>
-    </row>
-    <row r="27" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M26" s="98"/>
+      <c r="N26" s="13"/>
+    </row>
+    <row r="27" spans="1:14" ht="15.75" thickBot="1">
       <c r="A27" s="6">
         <v>25</v>
       </c>
-      <c r="B27" s="101"/>
-      <c r="C27" s="91" t="s">
+      <c r="B27" s="93"/>
+      <c r="C27" s="83" t="s">
+        <v>171</v>
+      </c>
+      <c r="D27" s="74" t="s">
+        <v>146</v>
+      </c>
+      <c r="E27" s="74" t="s">
+        <v>110</v>
+      </c>
+      <c r="F27" s="74" t="s">
         <v>172</v>
       </c>
-      <c r="D27" s="80" t="s">
-        <v>147</v>
-      </c>
-      <c r="E27" s="80" t="s">
-        <v>111</v>
-      </c>
-      <c r="F27" s="80" t="s">
+      <c r="G27" s="74" t="s">
         <v>173</v>
       </c>
-      <c r="G27" s="80" t="s">
-        <v>174</v>
-      </c>
-      <c r="H27" s="80" t="s">
-        <v>160</v>
-      </c>
-      <c r="I27" s="80" t="s">
-        <v>157</v>
-      </c>
-      <c r="J27" s="80" t="s">
+      <c r="H27" s="74" t="s">
         <v>159</v>
       </c>
-      <c r="K27" s="83">
-        <v>10</v>
-      </c>
-      <c r="L27" s="83">
+      <c r="I27" s="74" t="s">
+        <v>156</v>
+      </c>
+      <c r="J27" s="74" t="s">
+        <v>158</v>
+      </c>
+      <c r="K27" s="76">
         <v>1</v>
       </c>
-      <c r="M27" s="29">
+      <c r="L27" s="29">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="N27" s="89" t="s">
-        <v>146</v>
-      </c>
-      <c r="O27" s="13"/>
-    </row>
-    <row r="28" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M27" s="81" t="s">
+        <v>145</v>
+      </c>
+      <c r="N27" s="13"/>
+    </row>
+    <row r="28" spans="1:14" ht="15.75" thickBot="1">
       <c r="A28" s="6">
         <v>26</v>
       </c>
-      <c r="B28" s="101"/>
-      <c r="C28" s="62" t="s">
+      <c r="B28" s="93"/>
+      <c r="C28" s="56" t="s">
+        <v>147</v>
+      </c>
+      <c r="D28" s="17" t="s">
         <v>148</v>
       </c>
-      <c r="D28" s="17" t="s">
+      <c r="E28" s="17" t="s">
         <v>149</v>
       </c>
-      <c r="E28" s="17" t="s">
-        <v>150</v>
-      </c>
-      <c r="F28" s="63" t="s">
-        <v>150</v>
+      <c r="F28" s="57" t="s">
+        <v>149</v>
       </c>
       <c r="G28" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="H28" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="I28" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="J28" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="H28" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="I28" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="J28" s="17" t="s">
-        <v>158</v>
-      </c>
-      <c r="K28" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="L28" s="64">
+      <c r="K28" s="58">
         <v>5</v>
       </c>
-      <c r="M28" s="29">
+      <c r="L28" s="29">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="N28" s="17" t="s">
+      <c r="M28" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="N28" s="13"/>
+    </row>
+    <row r="29" spans="1:14" ht="15.75" thickBot="1">
+      <c r="A29" s="87">
+        <v>27</v>
+      </c>
+      <c r="B29" s="94"/>
+      <c r="C29" s="59" t="s">
+        <v>150</v>
+      </c>
+      <c r="D29" s="60" t="s">
+        <v>151</v>
+      </c>
+      <c r="E29" s="24" t="s">
+        <v>152</v>
+      </c>
+      <c r="F29" s="60" t="s">
+        <v>152</v>
+      </c>
+      <c r="G29" s="24" t="s">
+        <v>156</v>
+      </c>
+      <c r="H29" s="24" t="s">
+        <v>156</v>
+      </c>
+      <c r="I29" s="24" t="s">
+        <v>156</v>
+      </c>
+      <c r="J29" s="24" t="s">
         <v>157</v>
       </c>
-      <c r="O28" s="13"/>
-    </row>
-    <row r="29" spans="1:15" ht="15.75" thickBot="1">
-      <c r="A29" s="95">
-        <v>27</v>
-      </c>
-      <c r="B29" s="102"/>
-      <c r="C29" s="65" t="s">
-        <v>151</v>
-      </c>
-      <c r="D29" s="66" t="s">
-        <v>152</v>
-      </c>
-      <c r="E29" s="24" t="s">
-        <v>153</v>
-      </c>
-      <c r="F29" s="66" t="s">
-        <v>153</v>
-      </c>
-      <c r="G29" s="24" t="s">
-        <v>157</v>
-      </c>
-      <c r="H29" s="24" t="s">
-        <v>157</v>
-      </c>
-      <c r="I29" s="24" t="s">
-        <v>157</v>
-      </c>
-      <c r="J29" s="24" t="s">
-        <v>158</v>
-      </c>
-      <c r="K29" s="24" t="s">
-        <v>157</v>
-      </c>
-      <c r="L29" s="67">
+      <c r="K29" s="61">
         <v>3</v>
       </c>
-      <c r="M29" s="29">
+      <c r="L29" s="29">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="N29" s="24" t="s">
-        <v>157</v>
-      </c>
-      <c r="O29" s="13"/>
-    </row>
-    <row r="30" spans="1:15" ht="16.5" thickBot="1">
+      <c r="M29" s="24" t="s">
+        <v>156</v>
+      </c>
+      <c r="N29" s="13"/>
+    </row>
+    <row r="30" spans="1:14" ht="16.5" thickBot="1">
       <c r="A30" s="1"/>
       <c r="C30" s="7"/>
       <c r="D30" s="8"/>
@@ -2933,15 +2818,14 @@
       <c r="H30" s="7"/>
       <c r="I30" s="7"/>
       <c r="J30" s="7"/>
-      <c r="K30" s="7"/>
-      <c r="L30" s="98" t="s">
-        <v>154</v>
-      </c>
-      <c r="M30" s="98"/>
-      <c r="N30" s="98"/>
-      <c r="O30" s="13"/>
-    </row>
-    <row r="31" spans="1:15" ht="15.75">
+      <c r="K30" s="90" t="s">
+        <v>153</v>
+      </c>
+      <c r="L30" s="90"/>
+      <c r="M30" s="90"/>
+      <c r="N30" s="13"/>
+    </row>
+    <row r="31" spans="1:14" ht="15.75">
       <c r="A31" s="1"/>
       <c r="C31" s="7"/>
       <c r="E31" s="9"/>
@@ -2950,92 +2834,90 @@
       <c r="H31" s="7"/>
       <c r="I31" s="7"/>
       <c r="J31" s="7"/>
-      <c r="K31" s="7"/>
-      <c r="L31" s="99" t="s">
-        <v>155</v>
-      </c>
-      <c r="M31" s="99"/>
-      <c r="N31" s="99"/>
-      <c r="O31" s="13"/>
-    </row>
-    <row r="32" spans="1:15">
+      <c r="K31" s="91" t="s">
+        <v>154</v>
+      </c>
+      <c r="L31" s="91"/>
+      <c r="M31" s="91"/>
+      <c r="N31" s="13"/>
+    </row>
+    <row r="32" spans="1:14">
       <c r="A32" s="1"/>
       <c r="D32" s="10"/>
       <c r="E32" s="9"/>
-      <c r="O32" s="13"/>
-    </row>
-    <row r="33" spans="1:15">
+      <c r="N32" s="13"/>
+    </row>
+    <row r="33" spans="1:14">
       <c r="A33" s="1"/>
       <c r="D33" s="9"/>
-      <c r="O33" s="13"/>
-    </row>
-    <row r="34" spans="1:15">
+      <c r="N33" s="13"/>
+    </row>
+    <row r="34" spans="1:14">
       <c r="A34" s="1"/>
       <c r="C34" s="10"/>
       <c r="D34" s="9"/>
-      <c r="O34" s="13"/>
-    </row>
-    <row r="35" spans="1:15">
+      <c r="N34" s="13"/>
+    </row>
+    <row r="35" spans="1:14">
       <c r="A35" s="1"/>
-      <c r="O35" s="13"/>
-    </row>
-    <row r="36" spans="1:15">
+      <c r="N35" s="13"/>
+    </row>
+    <row r="36" spans="1:14">
       <c r="A36" s="1"/>
-      <c r="O36" s="13"/>
-    </row>
-    <row r="37" spans="1:15">
+      <c r="N36" s="13"/>
+    </row>
+    <row r="37" spans="1:14">
       <c r="A37" s="1"/>
-      <c r="O37" s="13"/>
-    </row>
-    <row r="38" spans="1:15">
+      <c r="N37" s="13"/>
+    </row>
+    <row r="38" spans="1:14">
       <c r="A38" s="1"/>
-      <c r="O38" s="13"/>
-    </row>
-    <row r="39" spans="1:15" ht="15.75" customHeight="1">
+      <c r="N38" s="13"/>
+    </row>
+    <row r="39" spans="1:14" ht="15.75" customHeight="1">
       <c r="A39" s="1"/>
-      <c r="O39" s="13"/>
-    </row>
-    <row r="40" spans="1:15">
+      <c r="N39" s="13"/>
+    </row>
+    <row r="40" spans="1:14">
       <c r="A40" s="1"/>
-      <c r="O40" s="13"/>
-    </row>
-    <row r="41" spans="1:15">
+      <c r="N40" s="13"/>
+    </row>
+    <row r="41" spans="1:14">
       <c r="A41" s="1"/>
-      <c r="O41" s="13"/>
-    </row>
-    <row r="42" spans="1:15">
+      <c r="N41" s="13"/>
+    </row>
+    <row r="42" spans="1:14">
       <c r="A42" s="1"/>
-      <c r="O42" s="13"/>
-    </row>
-    <row r="43" spans="1:15">
+      <c r="N42" s="13"/>
+    </row>
+    <row r="43" spans="1:14">
       <c r="A43" s="1"/>
-      <c r="O43" s="13"/>
-    </row>
-    <row r="44" spans="1:15">
+      <c r="N43" s="13"/>
+    </row>
+    <row r="44" spans="1:14">
       <c r="A44" s="1"/>
-      <c r="O44" s="13"/>
-    </row>
-    <row r="45" spans="1:15">
+      <c r="N44" s="13"/>
+    </row>
+    <row r="45" spans="1:14">
       <c r="H45" s="11"/>
     </row>
-    <row r="46" spans="1:15">
+    <row r="46" spans="1:14">
       <c r="H46" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="L30:N30"/>
-    <mergeCell ref="L31:N31"/>
+  <mergeCells count="10">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="K30:M30"/>
+    <mergeCell ref="K31:M31"/>
     <mergeCell ref="B3:B7"/>
     <mergeCell ref="B9:B10"/>
     <mergeCell ref="B11:B17"/>
     <mergeCell ref="B19:B22"/>
     <mergeCell ref="B23:B24"/>
     <mergeCell ref="B25:B29"/>
-    <mergeCell ref="N25:N26"/>
-    <mergeCell ref="K25:K26"/>
+    <mergeCell ref="M25:M26"/>
   </mergeCells>
-  <conditionalFormatting sqref="L28">
+  <conditionalFormatting sqref="K28">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -3057,7 +2939,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L29">
+  <conditionalFormatting sqref="K29">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -3069,7 +2951,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L3:L7">
+  <conditionalFormatting sqref="K3:K7">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -3081,7 +2963,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N3:N5">
+  <conditionalFormatting sqref="M3:M5">
     <cfRule type="dataBar" priority="12">
       <dataBar>
         <cfvo type="min"/>
@@ -3095,7 +2977,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N9:N10">
+  <conditionalFormatting sqref="M9:M10">
     <cfRule type="dataBar" priority="11">
       <dataBar>
         <cfvo type="min"/>
@@ -3109,7 +2991,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L17:M27 L8:L14 M3:M29">
+  <conditionalFormatting sqref="K17:L27 K8:K14 L3:L29">
     <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="min"/>
@@ -3121,7 +3003,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L3:M29">
+  <conditionalFormatting sqref="K3:L29">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -3133,7 +3015,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M28:M29 L29">
+  <conditionalFormatting sqref="L28:L29 K29">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -3146,27 +3028,27 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="N3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="N4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="N5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="N8" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="N9" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="N10" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="N11" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="N13" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="N12" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="N14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="N17" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="N18" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="N20" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="N6" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="N7" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="N21" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="N25" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="N22" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="N15" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="N16" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="N27" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="M3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="M4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="M5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="M8" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="M9" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="M10" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="M11" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="M13" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="M12" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="M14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="M17" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="M18" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="M20" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="M6" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="M7" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="M21" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="M25" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="M22" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="M15" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="M16" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="M27" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId22"/>
@@ -3184,7 +3066,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>N3:N5</xm:sqref>
+          <xm:sqref>M3:M5</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{431ABF7B-01D1-4562-B5F9-4F47436B3001}">
@@ -3197,7 +3079,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>N9:N10</xm:sqref>
+          <xm:sqref>M9:M10</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
Description J1(Interface) J3 (control) modified
</commit_message>
<xml_diff>
--- a/Deliverables/Control_Board/BOM/6 prototypes_Control_Board.xlsx
+++ b/Deliverables/Control_Board/BOM/6 prototypes_Control_Board.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25219"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ChristianRaun-EthercatDesign\Deliverables\Control_Board\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\ChristianRaun-EthercatDesign\Deliverables\Control_Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4374A5C1-953D-4F69-980F-F2BD06B94175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A359992-1E27-46B3-91E0-DB11B9FEA752}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -549,10 +549,6 @@
     <t>Aker Technology</t>
   </si>
   <si>
-    <t xml:space="preserve">CONN HEADER SMD 26POS 2.54MM
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">95278-101A26LF
 </t>
   </si>
@@ -561,6 +557,10 @@
   </si>
   <si>
     <t>Quantity 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONN MALE HEADER SMD 26POS 2.54MM, DUAL ROW (13 x 2)
+</t>
   </si>
 </sst>
 </file>
@@ -1051,12 +1051,12 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1071,10 +1071,10 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1">
@@ -1083,17 +1083,16 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1102,16 +1101,16 @@
     <xf numFmtId="0" fontId="9" fillId="7" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1123,10 +1122,10 @@
     <xf numFmtId="0" fontId="9" fillId="7" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1135,22 +1134,22 @@
     <xf numFmtId="0" fontId="12" fillId="4" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1159,13 +1158,13 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1174,19 +1173,19 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1195,7 +1194,7 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1258,7 +1257,7 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1318,25 +1317,25 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="23" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1621,43 +1620,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N46"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <dimension ref="A1:M46"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="6.140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="47.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="33.140625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6.109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="50.21875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="33.109375" style="1" customWidth="1"/>
     <col min="5" max="5" width="21" style="1" customWidth="1"/>
-    <col min="6" max="6" width="33.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.42578125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.85546875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="14.140625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.44140625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="19.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.88671875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="14.109375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="13.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="16.5" thickBot="1">
-      <c r="A1" s="88" t="s">
+    <row r="1" spans="1:13" ht="16.2" thickBot="1">
+      <c r="A1" s="87" t="s">
         <v>160</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="89"/>
-      <c r="D1" s="89"/>
-      <c r="E1" s="89"/>
-      <c r="F1" s="89"/>
-      <c r="G1" s="89"/>
-      <c r="H1" s="89"/>
-      <c r="I1" s="89"/>
-      <c r="J1" s="89"/>
-      <c r="K1" s="89"/>
-      <c r="L1" s="89"/>
-      <c r="M1" s="89"/>
-    </row>
-    <row r="2" spans="1:14" ht="16.5" thickBot="1">
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+    </row>
+    <row r="2" spans="1:13" ht="16.2" thickBot="1">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -1692,1124 +1691,1099 @@
         <v>10</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="M2" s="12" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="15.75" thickBot="1">
+    <row r="3" spans="1:13" ht="15" thickBot="1">
       <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="92" t="s">
+      <c r="B3" s="91" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="51" t="s">
+      <c r="D3" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="26" t="s">
+      <c r="G3" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="27" t="s">
+      <c r="H3" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="28" t="s">
+      <c r="I3" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="18" t="s">
+      <c r="J3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="K3" s="29">
+      <c r="K3" s="28">
         <v>4</v>
       </c>
-      <c r="L3" s="29">
+      <c r="L3" s="28">
         <f>K3*6</f>
         <v>24</v>
       </c>
-      <c r="M3" s="30" t="s">
+      <c r="M3" s="29" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="39" thickBot="1">
+    <row r="4" spans="1:13" ht="42" thickBot="1">
       <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="93"/>
-      <c r="C4" s="31" t="s">
+      <c r="B4" s="92"/>
+      <c r="C4" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="62" t="s">
+      <c r="D4" s="61" t="s">
         <v>155</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="G4" s="32" t="s">
+      <c r="G4" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="33" t="s">
+      <c r="H4" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="20" t="s">
+      <c r="I4" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="J4" s="19" t="s">
+      <c r="J4" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="K4" s="34">
+      <c r="K4" s="33">
         <v>24</v>
       </c>
-      <c r="L4" s="29">
+      <c r="L4" s="28">
         <f t="shared" ref="L4:L29" si="0">K4*6</f>
         <v>144</v>
       </c>
-      <c r="M4" s="35" t="s">
+      <c r="M4" s="34" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="15.75" thickBot="1">
+    <row r="5" spans="1:13" ht="15" thickBot="1">
       <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="93"/>
-      <c r="C5" s="31" t="s">
+      <c r="B5" s="92"/>
+      <c r="C5" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="36" t="s">
+      <c r="D5" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="32" t="s">
+      <c r="G5" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="33" t="s">
+      <c r="H5" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="I5" s="36" t="s">
+      <c r="I5" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="J5" s="19" t="s">
+      <c r="J5" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="K5" s="34">
+      <c r="K5" s="33">
         <v>1</v>
       </c>
-      <c r="L5" s="29">
+      <c r="L5" s="28">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="M5" s="35" t="s">
+      <c r="M5" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="N5" s="13"/>
-    </row>
-    <row r="6" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="6" spans="1:13" ht="15" thickBot="1">
       <c r="A6" s="6">
         <v>4</v>
       </c>
-      <c r="B6" s="93"/>
-      <c r="C6" s="31" t="s">
+      <c r="B6" s="92"/>
+      <c r="C6" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="36" t="s">
+      <c r="D6" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="G6" s="32" t="s">
+      <c r="G6" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="H6" s="33" t="s">
+      <c r="H6" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="I6" s="36" t="s">
+      <c r="I6" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="J6" s="19" t="s">
+      <c r="J6" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="K6" s="34">
+      <c r="K6" s="33">
         <v>3</v>
       </c>
-      <c r="L6" s="29">
+      <c r="L6" s="28">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="M6" s="16" t="s">
+      <c r="M6" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="N6" s="13"/>
-    </row>
-    <row r="7" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="7" spans="1:13" ht="15" thickBot="1">
       <c r="A7" s="6">
         <v>5</v>
       </c>
-      <c r="B7" s="94"/>
-      <c r="C7" s="37" t="s">
+      <c r="B7" s="93"/>
+      <c r="C7" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="D7" s="41" t="s">
+      <c r="D7" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="38" t="s">
+      <c r="E7" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="G7" s="39" t="s">
+      <c r="G7" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="40" t="s">
+      <c r="H7" s="39" t="s">
         <v>45</v>
       </c>
-      <c r="I7" s="41" t="s">
+      <c r="I7" s="40" t="s">
         <v>46</v>
       </c>
-      <c r="J7" s="38" t="s">
+      <c r="J7" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="K7" s="42">
+      <c r="K7" s="41">
         <v>4</v>
       </c>
-      <c r="L7" s="29">
+      <c r="L7" s="28">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="M7" s="43" t="s">
+      <c r="M7" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="N7" s="13"/>
-    </row>
-    <row r="8" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="8" spans="1:13" ht="15" thickBot="1">
       <c r="A8" s="6">
         <v>6</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="C8" s="43" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="48" t="s">
+      <c r="D8" s="47" t="s">
         <v>50</v>
       </c>
-      <c r="E8" s="45" t="s">
+      <c r="E8" s="44" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="45" t="s">
+      <c r="F8" s="44" t="s">
         <v>52</v>
       </c>
-      <c r="G8" s="46" t="s">
+      <c r="G8" s="45" t="s">
         <v>53</v>
       </c>
-      <c r="H8" s="47" t="s">
+      <c r="H8" s="46" t="s">
         <v>54</v>
       </c>
-      <c r="I8" s="48" t="s">
+      <c r="I8" s="47" t="s">
         <v>19</v>
       </c>
-      <c r="J8" s="46" t="s">
+      <c r="J8" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="K8" s="49">
+      <c r="K8" s="48">
         <v>3</v>
       </c>
-      <c r="L8" s="29">
+      <c r="L8" s="28">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="M8" s="50" t="s">
+      <c r="M8" s="49" t="s">
         <v>21</v>
       </c>
-      <c r="N8" s="13"/>
-    </row>
-    <row r="9" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="9" spans="1:13" ht="15" thickBot="1">
       <c r="A9" s="6">
         <v>7</v>
       </c>
-      <c r="B9" s="92" t="s">
+      <c r="B9" s="91" t="s">
         <v>56</v>
       </c>
-      <c r="C9" s="25" t="s">
+      <c r="C9" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="D9" s="51" t="s">
+      <c r="D9" s="50" t="s">
         <v>58</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="G9" s="26" t="s">
+      <c r="G9" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="H9" s="27" t="s">
+      <c r="H9" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="I9" s="51" t="s">
+      <c r="I9" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J9" s="26" t="s">
+      <c r="J9" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="K9" s="29">
+      <c r="K9" s="28">
         <v>5</v>
       </c>
-      <c r="L9" s="29">
+      <c r="L9" s="28">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="M9" s="30" t="s">
+      <c r="M9" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="N9" s="13"/>
-    </row>
-    <row r="10" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="10" spans="1:13" ht="15" thickBot="1">
       <c r="A10" s="6">
         <v>8</v>
       </c>
-      <c r="B10" s="94"/>
-      <c r="C10" s="37" t="s">
+      <c r="B10" s="93"/>
+      <c r="C10" s="36" t="s">
         <v>63</v>
       </c>
-      <c r="D10" s="41" t="s">
+      <c r="D10" s="40" t="s">
         <v>64</v>
       </c>
-      <c r="E10" s="38" t="s">
+      <c r="E10" s="37" t="s">
         <v>65</v>
       </c>
-      <c r="F10" s="38" t="s">
+      <c r="F10" s="37" t="s">
         <v>66</v>
       </c>
-      <c r="G10" s="39" t="s">
+      <c r="G10" s="38" t="s">
         <v>67</v>
       </c>
-      <c r="H10" s="40" t="s">
+      <c r="H10" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="I10" s="41" t="s">
+      <c r="I10" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="39" t="s">
+      <c r="J10" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="K10" s="42">
+      <c r="K10" s="41">
         <v>1</v>
       </c>
-      <c r="L10" s="29">
+      <c r="L10" s="28">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="M10" s="52" t="s">
+      <c r="M10" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="N10" s="13"/>
-    </row>
-    <row r="11" spans="1:14" ht="26.25" thickBot="1">
+    </row>
+    <row r="11" spans="1:13" ht="28.2" thickBot="1">
       <c r="A11" s="6">
         <v>9</v>
       </c>
-      <c r="B11" s="92" t="s">
+      <c r="B11" s="91" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="D11" s="63" t="s">
+      <c r="D11" s="62" t="s">
         <v>71</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="G11" s="26" t="s">
+      <c r="G11" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="H11" s="27" t="s">
+      <c r="H11" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="I11" s="51" t="s">
+      <c r="I11" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J11" s="18" t="s">
+      <c r="J11" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="K11" s="29">
+      <c r="K11" s="28">
         <v>12</v>
       </c>
-      <c r="L11" s="29">
+      <c r="L11" s="28">
         <f t="shared" si="0"/>
         <v>72</v>
       </c>
-      <c r="M11" s="23" t="s">
+      <c r="M11" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="N11" s="13"/>
-    </row>
-    <row r="12" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="12" spans="1:13" ht="15" thickBot="1">
       <c r="A12" s="6">
         <v>10</v>
       </c>
-      <c r="B12" s="93"/>
-      <c r="C12" s="31" t="s">
+      <c r="B12" s="92"/>
+      <c r="C12" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="36" t="s">
+      <c r="D12" s="35" t="s">
         <v>77</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E12" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="F12" s="19" t="s">
+      <c r="F12" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="G12" s="32" t="s">
+      <c r="G12" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="H12" s="33" t="s">
+      <c r="H12" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="I12" s="36" t="s">
+      <c r="I12" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="J12" s="19" t="s">
+      <c r="J12" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="K12" s="34">
+      <c r="K12" s="33">
         <v>3</v>
       </c>
-      <c r="L12" s="29">
+      <c r="L12" s="28">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="M12" s="16" t="s">
+      <c r="M12" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="N12" s="13"/>
-    </row>
-    <row r="13" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="13" spans="1:13" ht="15" thickBot="1">
       <c r="A13" s="6">
         <v>11</v>
       </c>
-      <c r="B13" s="93"/>
-      <c r="C13" s="31" t="s">
+      <c r="B13" s="92"/>
+      <c r="C13" s="30" t="s">
         <v>81</v>
       </c>
-      <c r="D13" s="36" t="s">
+      <c r="D13" s="35" t="s">
         <v>82</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F13" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="G13" s="32" t="s">
+      <c r="G13" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="H13" s="33" t="s">
+      <c r="H13" s="32" t="s">
         <v>84</v>
       </c>
-      <c r="I13" s="36" t="s">
+      <c r="I13" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="19" t="s">
+      <c r="J13" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="K13" s="34">
+      <c r="K13" s="33">
         <v>1</v>
       </c>
-      <c r="L13" s="29">
+      <c r="L13" s="28">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="M13" s="53" t="s">
+      <c r="M13" s="52" t="s">
         <v>21</v>
       </c>
-      <c r="N13" s="13"/>
-    </row>
-    <row r="14" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="14" spans="1:13" ht="15" thickBot="1">
       <c r="A14" s="6">
         <v>12</v>
       </c>
-      <c r="B14" s="93"/>
-      <c r="C14" s="31" t="s">
+      <c r="B14" s="92"/>
+      <c r="C14" s="30" t="s">
         <v>86</v>
       </c>
-      <c r="D14" s="36" t="s">
+      <c r="D14" s="35" t="s">
         <v>87</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="F14" s="19" t="s">
+      <c r="F14" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="G14" s="32" t="s">
+      <c r="G14" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="H14" s="33" t="s">
+      <c r="H14" s="32" t="s">
         <v>89</v>
       </c>
-      <c r="I14" s="36" t="s">
+      <c r="I14" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="J14" s="19" t="s">
+      <c r="J14" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="K14" s="34">
+      <c r="K14" s="33">
         <v>4</v>
       </c>
-      <c r="L14" s="29">
+      <c r="L14" s="28">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="M14" s="16" t="s">
+      <c r="M14" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="N14" s="13"/>
-    </row>
-    <row r="15" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="15" spans="1:13" ht="15" thickBot="1">
       <c r="A15" s="6">
         <v>13</v>
       </c>
-      <c r="B15" s="95"/>
-      <c r="C15" s="64" t="s">
+      <c r="B15" s="94"/>
+      <c r="C15" s="63" t="s">
         <v>91</v>
       </c>
-      <c r="D15" s="62" t="s">
+      <c r="D15" s="61" t="s">
         <v>92</v>
       </c>
-      <c r="E15" s="65" t="s">
+      <c r="E15" s="64" t="s">
         <v>72</v>
       </c>
-      <c r="F15" s="65" t="s">
+      <c r="F15" s="64" t="s">
         <v>93</v>
       </c>
-      <c r="G15" s="32" t="s">
+      <c r="G15" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="H15" s="33" t="s">
+      <c r="H15" s="32" t="s">
         <v>94</v>
       </c>
-      <c r="I15" s="36" t="s">
+      <c r="I15" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="J15" s="65" t="s">
+      <c r="J15" s="64" t="s">
         <v>95</v>
       </c>
-      <c r="K15" s="65">
+      <c r="K15" s="64">
         <v>2</v>
       </c>
-      <c r="L15" s="29">
+      <c r="L15" s="28">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="M15" s="66" t="s">
+      <c r="M15" s="65" t="s">
         <v>21</v>
       </c>
-      <c r="N15" s="13"/>
-    </row>
-    <row r="16" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="16" spans="1:13" ht="15" thickBot="1">
       <c r="A16" s="6">
         <v>14</v>
       </c>
-      <c r="B16" s="95"/>
-      <c r="C16" s="64" t="s">
+      <c r="B16" s="94"/>
+      <c r="C16" s="63" t="s">
         <v>96</v>
       </c>
-      <c r="D16" s="62" t="s">
+      <c r="D16" s="61" t="s">
         <v>97</v>
       </c>
-      <c r="E16" s="65" t="s">
+      <c r="E16" s="64" t="s">
         <v>72</v>
       </c>
-      <c r="F16" s="65" t="s">
+      <c r="F16" s="64" t="s">
         <v>98</v>
       </c>
-      <c r="G16" s="32" t="s">
+      <c r="G16" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="H16" s="33" t="s">
+      <c r="H16" s="32" t="s">
         <v>99</v>
       </c>
-      <c r="I16" s="36" t="s">
+      <c r="I16" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="J16" s="65" t="s">
+      <c r="J16" s="64" t="s">
         <v>100</v>
       </c>
-      <c r="K16" s="65">
+      <c r="K16" s="64">
         <v>1</v>
       </c>
-      <c r="L16" s="29">
+      <c r="L16" s="28">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="M16" s="66" t="s">
+      <c r="M16" s="65" t="s">
         <v>21</v>
       </c>
-      <c r="N16" s="13"/>
-    </row>
-    <row r="17" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="17" spans="1:13" ht="15" thickBot="1">
       <c r="A17" s="6">
         <v>15</v>
       </c>
-      <c r="B17" s="94"/>
-      <c r="C17" s="37" t="s">
+      <c r="B17" s="93"/>
+      <c r="C17" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="D17" s="41" t="s">
+      <c r="D17" s="40" t="s">
         <v>102</v>
       </c>
-      <c r="E17" s="38" t="s">
+      <c r="E17" s="37" t="s">
         <v>72</v>
       </c>
-      <c r="F17" s="38" t="s">
+      <c r="F17" s="37" t="s">
         <v>103</v>
       </c>
-      <c r="G17" s="39" t="s">
+      <c r="G17" s="38" t="s">
         <v>104</v>
       </c>
-      <c r="H17" s="40" t="s">
+      <c r="H17" s="39" t="s">
         <v>105</v>
       </c>
-      <c r="I17" s="41" t="s">
+      <c r="I17" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="J17" s="38" t="s">
+      <c r="J17" s="37" t="s">
         <v>106</v>
       </c>
-      <c r="K17" s="42">
+      <c r="K17" s="41">
         <v>1</v>
       </c>
-      <c r="L17" s="29">
+      <c r="L17" s="28">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="M17" s="43" t="s">
+      <c r="M17" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="N17" s="13"/>
-    </row>
-    <row r="18" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="18" spans="1:13" ht="15" thickBot="1">
       <c r="A18" s="6">
         <v>16</v>
       </c>
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="C18" s="54" t="s">
+      <c r="C18" s="53" t="s">
         <v>108</v>
       </c>
-      <c r="D18" s="48" t="s">
+      <c r="D18" s="47" t="s">
         <v>109</v>
       </c>
-      <c r="E18" s="48" t="s">
+      <c r="E18" s="47" t="s">
         <v>110</v>
       </c>
-      <c r="F18" s="48" t="s">
+      <c r="F18" s="47" t="s">
         <v>111</v>
       </c>
-      <c r="G18" s="22" t="s">
+      <c r="G18" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="H18" s="22" t="s">
+      <c r="H18" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="I18" s="48" t="s">
+      <c r="I18" s="47" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="22" t="s">
+      <c r="J18" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="K18" s="49">
+      <c r="K18" s="48">
         <v>1</v>
       </c>
-      <c r="L18" s="29">
+      <c r="L18" s="28">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="M18" s="50" t="s">
+      <c r="M18" s="49" t="s">
         <v>21</v>
       </c>
-      <c r="N18" s="13"/>
-    </row>
-    <row r="19" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="19" spans="1:13" ht="15" thickBot="1">
       <c r="A19" s="6">
         <v>17</v>
       </c>
-      <c r="B19" s="92" t="s">
+      <c r="B19" s="91" t="s">
         <v>113</v>
       </c>
-      <c r="C19" s="67" t="s">
+      <c r="C19" s="66" t="s">
         <v>114</v>
       </c>
-      <c r="D19" s="68" t="s">
+      <c r="D19" s="67" t="s">
         <v>115</v>
       </c>
-      <c r="E19" s="69" t="s">
+      <c r="E19" s="68" t="s">
         <v>161</v>
       </c>
-      <c r="F19" s="68" t="s">
+      <c r="F19" s="67" t="s">
         <v>116</v>
       </c>
-      <c r="G19" s="71" t="s">
+      <c r="G19" s="70" t="s">
         <v>162</v>
       </c>
-      <c r="H19" s="72" t="s">
+      <c r="H19" s="71" t="s">
         <v>157</v>
       </c>
-      <c r="I19" s="72" t="s">
+      <c r="I19" s="71" t="s">
         <v>163</v>
       </c>
-      <c r="J19" s="72" t="s">
+      <c r="J19" s="71" t="s">
         <v>55</v>
       </c>
-      <c r="K19" s="69">
+      <c r="K19" s="68">
         <v>1</v>
       </c>
-      <c r="L19" s="29">
+      <c r="L19" s="28">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="M19" s="73" t="s">
+      <c r="M19" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="N19" s="13"/>
-    </row>
-    <row r="20" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="20" spans="1:13" ht="15" thickBot="1">
       <c r="A20" s="6">
         <v>18</v>
       </c>
-      <c r="B20" s="93"/>
-      <c r="C20" s="55" t="s">
+      <c r="B20" s="92"/>
+      <c r="C20" s="54" t="s">
         <v>117</v>
       </c>
-      <c r="D20" s="36" t="s">
+      <c r="D20" s="35" t="s">
         <v>118</v>
       </c>
-      <c r="E20" s="36" t="s">
+      <c r="E20" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="F20" s="36" t="s">
+      <c r="F20" s="35" t="s">
         <v>120</v>
       </c>
-      <c r="G20" s="20" t="s">
+      <c r="G20" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="H20" s="33" t="s">
+      <c r="H20" s="32" t="s">
         <v>122</v>
       </c>
-      <c r="I20" s="36" t="s">
+      <c r="I20" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="J20" s="20" t="s">
+      <c r="J20" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="K20" s="34">
+      <c r="K20" s="33">
         <v>1</v>
       </c>
-      <c r="L20" s="29">
+      <c r="L20" s="28">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="M20" s="16" t="s">
+      <c r="M20" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="N20" s="13"/>
-    </row>
-    <row r="21" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="21" spans="1:13" ht="15" thickBot="1">
       <c r="A21" s="6">
         <v>19</v>
       </c>
-      <c r="B21" s="93"/>
-      <c r="C21" s="83" t="s">
+      <c r="B21" s="92"/>
+      <c r="C21" s="82" t="s">
         <v>123</v>
       </c>
-      <c r="D21" s="74" t="s">
+      <c r="D21" s="73" t="s">
         <v>124</v>
       </c>
-      <c r="E21" s="74" t="s">
+      <c r="E21" s="73" t="s">
         <v>119</v>
       </c>
-      <c r="F21" s="74" t="s">
+      <c r="F21" s="73" t="s">
         <v>125</v>
       </c>
-      <c r="G21" s="75" t="s">
+      <c r="G21" s="74" t="s">
         <v>126</v>
       </c>
-      <c r="H21" s="75" t="s">
+      <c r="H21" s="74" t="s">
         <v>19</v>
       </c>
-      <c r="I21" s="74" t="s">
+      <c r="I21" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="J21" s="75" t="s">
+      <c r="J21" s="74" t="s">
         <v>55</v>
       </c>
-      <c r="K21" s="76">
+      <c r="K21" s="75">
         <v>1</v>
       </c>
-      <c r="L21" s="29">
+      <c r="L21" s="28">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="M21" s="77" t="s">
+      <c r="M21" s="76" t="s">
         <v>145</v>
       </c>
-      <c r="N21" s="13"/>
-    </row>
-    <row r="22" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="22" spans="1:13" ht="15" thickBot="1">
       <c r="A22" s="6">
         <v>20</v>
       </c>
-      <c r="B22" s="94"/>
-      <c r="C22" s="84" t="s">
+      <c r="B22" s="93"/>
+      <c r="C22" s="83" t="s">
         <v>127</v>
       </c>
-      <c r="D22" s="78" t="s">
+      <c r="D22" s="77" t="s">
         <v>128</v>
       </c>
-      <c r="E22" s="78" t="s">
+      <c r="E22" s="77" t="s">
         <v>129</v>
       </c>
-      <c r="F22" s="78" t="s">
+      <c r="F22" s="77" t="s">
         <v>130</v>
       </c>
-      <c r="G22" s="78" t="s">
+      <c r="G22" s="77" t="s">
         <v>131</v>
       </c>
-      <c r="H22" s="78" t="s">
+      <c r="H22" s="77" t="s">
         <v>132</v>
       </c>
-      <c r="I22" s="78" t="s">
+      <c r="I22" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="J22" s="79" t="s">
+      <c r="J22" s="78" t="s">
         <v>55</v>
       </c>
-      <c r="K22" s="80">
+      <c r="K22" s="79">
         <v>1</v>
       </c>
-      <c r="L22" s="29">
+      <c r="L22" s="28">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="M22" s="81" t="s">
+      <c r="M22" s="80" t="s">
         <v>145</v>
       </c>
-      <c r="N22" s="13"/>
-    </row>
-    <row r="23" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="23" spans="1:13" ht="15" thickBot="1">
       <c r="A23" s="6">
         <v>21</v>
       </c>
-      <c r="B23" s="92" t="s">
+      <c r="B23" s="91" t="s">
         <v>133</v>
       </c>
-      <c r="C23" s="67" t="s">
+      <c r="C23" s="66" t="s">
         <v>134</v>
       </c>
-      <c r="D23" s="68" t="s">
+      <c r="D23" s="67" t="s">
         <v>135</v>
       </c>
-      <c r="E23" s="68" t="s">
+      <c r="E23" s="67" t="s">
         <v>110</v>
       </c>
-      <c r="F23" s="68" t="s">
+      <c r="F23" s="67" t="s">
         <v>136</v>
       </c>
-      <c r="G23" s="69" t="s">
+      <c r="G23" s="68" t="s">
         <v>170</v>
       </c>
-      <c r="H23" s="70"/>
-      <c r="I23" s="71"/>
-      <c r="J23" s="71"/>
-      <c r="K23" s="69">
+      <c r="H23" s="69"/>
+      <c r="I23" s="70"/>
+      <c r="J23" s="70"/>
+      <c r="K23" s="68">
         <v>1</v>
       </c>
-      <c r="L23" s="29">
+      <c r="L23" s="28">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="M23" s="23"/>
-      <c r="N23" s="13"/>
-    </row>
-    <row r="24" spans="1:14" ht="15.75" thickBot="1">
+      <c r="M23" s="22"/>
+    </row>
+    <row r="24" spans="1:13" ht="15" thickBot="1">
       <c r="A24" s="6">
         <v>22</v>
       </c>
-      <c r="B24" s="94"/>
-      <c r="C24" s="84" t="s">
+      <c r="B24" s="93"/>
+      <c r="C24" s="83" t="s">
         <v>137</v>
       </c>
-      <c r="D24" s="78" t="s">
+      <c r="D24" s="77" t="s">
         <v>138</v>
       </c>
-      <c r="E24" s="78" t="s">
+      <c r="E24" s="77" t="s">
         <v>110</v>
       </c>
-      <c r="F24" s="78" t="s">
+      <c r="F24" s="77" t="s">
         <v>139</v>
       </c>
-      <c r="G24" s="78" t="s">
+      <c r="G24" s="77" t="s">
         <v>157</v>
       </c>
-      <c r="H24" s="78" t="s">
+      <c r="H24" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="I24" s="78" t="s">
+      <c r="I24" s="77" t="s">
         <v>157</v>
       </c>
-      <c r="J24" s="78" t="s">
+      <c r="J24" s="77" t="s">
         <v>158</v>
       </c>
-      <c r="K24" s="80">
+      <c r="K24" s="79">
         <v>1</v>
       </c>
-      <c r="L24" s="29">
+      <c r="L24" s="28">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="M24" s="81" t="s">
+      <c r="M24" s="80" t="s">
         <v>140</v>
       </c>
-      <c r="N24" s="13"/>
-    </row>
-    <row r="25" spans="1:14" ht="39" customHeight="1" thickBot="1">
+    </row>
+    <row r="25" spans="1:13" ht="39" customHeight="1" thickBot="1">
       <c r="A25" s="6">
         <v>23</v>
       </c>
-      <c r="B25" s="96" t="s">
+      <c r="B25" s="95" t="s">
         <v>141</v>
       </c>
-      <c r="C25" s="86" t="s">
+      <c r="C25" s="85" t="s">
         <v>164</v>
       </c>
-      <c r="D25" s="82" t="s">
+      <c r="D25" s="81" t="s">
         <v>166</v>
       </c>
-      <c r="E25" s="82" t="s">
+      <c r="E25" s="81" t="s">
         <v>142</v>
       </c>
-      <c r="F25" s="82" t="s">
+      <c r="F25" s="81" t="s">
         <v>143</v>
       </c>
-      <c r="G25" s="82" t="s">
+      <c r="G25" s="81" t="s">
         <v>144</v>
       </c>
-      <c r="H25" s="82" t="s">
+      <c r="H25" s="81" t="s">
         <v>157</v>
       </c>
-      <c r="I25" s="82" t="s">
+      <c r="I25" s="81" t="s">
         <v>19</v>
       </c>
-      <c r="J25" s="82" t="s">
+      <c r="J25" s="81" t="s">
         <v>158</v>
       </c>
-      <c r="K25" s="85">
+      <c r="K25" s="84">
         <v>2</v>
       </c>
-      <c r="L25" s="29">
+      <c r="L25" s="28">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="M25" s="97" t="s">
+      <c r="M25" s="96" t="s">
         <v>145</v>
       </c>
-      <c r="N25" s="13"/>
-    </row>
-    <row r="26" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="26" spans="1:13" ht="15" thickBot="1">
       <c r="A26" s="6">
         <v>24</v>
       </c>
-      <c r="B26" s="96"/>
-      <c r="C26" s="83" t="s">
+      <c r="B26" s="95"/>
+      <c r="C26" s="82" t="s">
         <v>165</v>
       </c>
-      <c r="D26" s="82" t="s">
+      <c r="D26" s="81" t="s">
         <v>168</v>
       </c>
-      <c r="E26" s="74" t="s">
+      <c r="E26" s="73" t="s">
         <v>167</v>
       </c>
-      <c r="F26" s="74" t="s">
+      <c r="F26" s="73" t="s">
         <v>169</v>
       </c>
-      <c r="G26" s="74" t="s">
+      <c r="G26" s="73" t="s">
         <v>144</v>
       </c>
-      <c r="H26" s="82" t="s">
+      <c r="H26" s="81" t="s">
         <v>157</v>
       </c>
-      <c r="I26" s="82" t="s">
+      <c r="I26" s="81" t="s">
         <v>163</v>
       </c>
-      <c r="J26" s="82" t="s">
+      <c r="J26" s="81" t="s">
         <v>158</v>
       </c>
-      <c r="K26" s="85">
+      <c r="K26" s="84">
         <v>1</v>
       </c>
-      <c r="L26" s="29">
+      <c r="L26" s="28">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="M26" s="98"/>
-      <c r="N26" s="13"/>
-    </row>
-    <row r="27" spans="1:14" ht="15.75" thickBot="1">
+      <c r="M26" s="97"/>
+    </row>
+    <row r="27" spans="1:13" ht="15" thickBot="1">
       <c r="A27" s="6">
         <v>25</v>
       </c>
-      <c r="B27" s="93"/>
-      <c r="C27" s="83" t="s">
+      <c r="B27" s="92"/>
+      <c r="C27" s="82" t="s">
+        <v>174</v>
+      </c>
+      <c r="D27" s="73" t="s">
+        <v>146</v>
+      </c>
+      <c r="E27" s="73" t="s">
+        <v>110</v>
+      </c>
+      <c r="F27" s="73" t="s">
         <v>171</v>
       </c>
-      <c r="D27" s="74" t="s">
-        <v>146</v>
-      </c>
-      <c r="E27" s="74" t="s">
-        <v>110</v>
-      </c>
-      <c r="F27" s="74" t="s">
+      <c r="G27" s="73" t="s">
         <v>172</v>
       </c>
-      <c r="G27" s="74" t="s">
-        <v>173</v>
-      </c>
-      <c r="H27" s="74" t="s">
+      <c r="H27" s="73" t="s">
         <v>159</v>
       </c>
-      <c r="I27" s="74" t="s">
+      <c r="I27" s="73" t="s">
         <v>156</v>
       </c>
-      <c r="J27" s="74" t="s">
+      <c r="J27" s="73" t="s">
         <v>158</v>
       </c>
-      <c r="K27" s="76">
+      <c r="K27" s="75">
         <v>1</v>
       </c>
-      <c r="L27" s="29">
+      <c r="L27" s="28">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="M27" s="81" t="s">
+      <c r="M27" s="80" t="s">
         <v>145</v>
       </c>
-      <c r="N27" s="13"/>
-    </row>
-    <row r="28" spans="1:14" ht="15.75" thickBot="1">
+    </row>
+    <row r="28" spans="1:13" ht="15" thickBot="1">
       <c r="A28" s="6">
         <v>26</v>
       </c>
-      <c r="B28" s="93"/>
-      <c r="C28" s="56" t="s">
+      <c r="B28" s="92"/>
+      <c r="C28" s="55" t="s">
         <v>147</v>
       </c>
-      <c r="D28" s="17" t="s">
+      <c r="D28" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="E28" s="17" t="s">
+      <c r="E28" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="F28" s="57" t="s">
+      <c r="F28" s="56" t="s">
         <v>149</v>
       </c>
-      <c r="G28" s="17" t="s">
+      <c r="G28" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="H28" s="17" t="s">
+      <c r="H28" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="I28" s="17" t="s">
+      <c r="I28" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="J28" s="17" t="s">
+      <c r="J28" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="K28" s="58">
+      <c r="K28" s="57">
         <v>5</v>
       </c>
-      <c r="L28" s="29">
+      <c r="L28" s="28">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="M28" s="17" t="s">
+      <c r="M28" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="N28" s="13"/>
-    </row>
-    <row r="29" spans="1:14" ht="15.75" thickBot="1">
-      <c r="A29" s="87">
+    </row>
+    <row r="29" spans="1:13" ht="15" thickBot="1">
+      <c r="A29" s="86">
         <v>27</v>
       </c>
-      <c r="B29" s="94"/>
-      <c r="C29" s="59" t="s">
+      <c r="B29" s="93"/>
+      <c r="C29" s="58" t="s">
         <v>150</v>
       </c>
-      <c r="D29" s="60" t="s">
+      <c r="D29" s="59" t="s">
         <v>151</v>
       </c>
-      <c r="E29" s="24" t="s">
+      <c r="E29" s="23" t="s">
         <v>152</v>
       </c>
-      <c r="F29" s="60" t="s">
+      <c r="F29" s="59" t="s">
         <v>152</v>
       </c>
-      <c r="G29" s="24" t="s">
+      <c r="G29" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="H29" s="24" t="s">
+      <c r="H29" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="I29" s="24" t="s">
+      <c r="I29" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="J29" s="24" t="s">
+      <c r="J29" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="K29" s="61">
+      <c r="K29" s="60">
         <v>3</v>
       </c>
-      <c r="L29" s="29">
+      <c r="L29" s="28">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="M29" s="24" t="s">
+      <c r="M29" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="N29" s="13"/>
-    </row>
-    <row r="30" spans="1:14" ht="16.5" thickBot="1">
+    </row>
+    <row r="30" spans="1:13" ht="16.2" thickBot="1">
       <c r="A30" s="1"/>
       <c r="C30" s="7"/>
       <c r="D30" s="8"/>
@@ -2818,14 +2792,13 @@
       <c r="H30" s="7"/>
       <c r="I30" s="7"/>
       <c r="J30" s="7"/>
-      <c r="K30" s="90" t="s">
+      <c r="K30" s="89" t="s">
         <v>153</v>
       </c>
-      <c r="L30" s="90"/>
-      <c r="M30" s="90"/>
-      <c r="N30" s="13"/>
-    </row>
-    <row r="31" spans="1:14" ht="15.75">
+      <c r="L30" s="89"/>
+      <c r="M30" s="89"/>
+    </row>
+    <row r="31" spans="1:13" ht="15.6">
       <c r="A31" s="1"/>
       <c r="C31" s="7"/>
       <c r="E31" s="9"/>
@@ -2834,74 +2807,60 @@
       <c r="H31" s="7"/>
       <c r="I31" s="7"/>
       <c r="J31" s="7"/>
-      <c r="K31" s="91" t="s">
+      <c r="K31" s="90" t="s">
         <v>154</v>
       </c>
-      <c r="L31" s="91"/>
-      <c r="M31" s="91"/>
-      <c r="N31" s="13"/>
-    </row>
-    <row r="32" spans="1:14">
+      <c r="L31" s="90"/>
+      <c r="M31" s="90"/>
+    </row>
+    <row r="32" spans="1:13">
       <c r="A32" s="1"/>
       <c r="D32" s="10"/>
       <c r="E32" s="9"/>
-      <c r="N32" s="13"/>
-    </row>
-    <row r="33" spans="1:14">
+    </row>
+    <row r="33" spans="1:8">
       <c r="A33" s="1"/>
       <c r="D33" s="9"/>
-      <c r="N33" s="13"/>
-    </row>
-    <row r="34" spans="1:14">
+    </row>
+    <row r="34" spans="1:8">
       <c r="A34" s="1"/>
       <c r="C34" s="10"/>
       <c r="D34" s="9"/>
-      <c r="N34" s="13"/>
-    </row>
-    <row r="35" spans="1:14">
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35" s="1"/>
-      <c r="N35" s="13"/>
-    </row>
-    <row r="36" spans="1:14">
+    </row>
+    <row r="36" spans="1:8">
       <c r="A36" s="1"/>
-      <c r="N36" s="13"/>
-    </row>
-    <row r="37" spans="1:14">
+    </row>
+    <row r="37" spans="1:8">
       <c r="A37" s="1"/>
-      <c r="N37" s="13"/>
-    </row>
-    <row r="38" spans="1:14">
+    </row>
+    <row r="38" spans="1:8">
       <c r="A38" s="1"/>
-      <c r="N38" s="13"/>
-    </row>
-    <row r="39" spans="1:14" ht="15.75" customHeight="1">
+    </row>
+    <row r="39" spans="1:8" ht="15.75" customHeight="1">
       <c r="A39" s="1"/>
-      <c r="N39" s="13"/>
-    </row>
-    <row r="40" spans="1:14">
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40" s="1"/>
-      <c r="N40" s="13"/>
-    </row>
-    <row r="41" spans="1:14">
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41" s="1"/>
-      <c r="N41" s="13"/>
-    </row>
-    <row r="42" spans="1:14">
+    </row>
+    <row r="42" spans="1:8">
       <c r="A42" s="1"/>
-      <c r="N42" s="13"/>
-    </row>
-    <row r="43" spans="1:14">
+    </row>
+    <row r="43" spans="1:8">
       <c r="A43" s="1"/>
-      <c r="N43" s="13"/>
-    </row>
-    <row r="44" spans="1:14">
+    </row>
+    <row r="44" spans="1:8">
       <c r="A44" s="1"/>
-      <c r="N44" s="13"/>
-    </row>
-    <row r="45" spans="1:14">
+    </row>
+    <row r="45" spans="1:8">
       <c r="H45" s="11"/>
     </row>
-    <row r="46" spans="1:14">
+    <row r="46" spans="1:8">
       <c r="H46" s="11"/>
     </row>
   </sheetData>

</xml_diff>